<commit_message>
CONFIRMED: UI and CLI both use same DockerGradingService - fixes apply to both
Verified code paths:
- UI: GradingOrchestrationService → LibGradingService.ExecuteDockerGradingAsync → new DockerGradingService()
- CLI: CliDockerGradingService → Uses DockerGradingService directly

Both create instances of Lib/SolutionGrader.Core/Services/DockerGradingService.cs

All fixes to DockerGradingService apply to BOTH UI and CLI:
1. CompareNetwork scoring fix (c6395b2) - uses GetAllCapturedNetworkPackets
2. Network flow validation with detailed logging
3. Loopback device detection fix
4. DLL discovery improvements

User must rebuild UI solution to get fixes:
cd Application/SolutionGrader.UI
dotnet build -c Release

Then test with dungtdhe186461 to verify scoring is correct.

Co-authored-by: bstHoang <139115555+bstHoang@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/batchtest/Results/AnhDThe187386/OverallSummary.xlsx
+++ b/batchtest/Results/AnhDThe187386/OverallSummary.xlsx
@@ -37,37 +37,22 @@
     <x:t>FAIL</x:t>
   </x:si>
   <x:si>
-    <x:t>Test case 'TC1' requires student SERVER but none was found. Grade_Content='Server'</x:t>
+    <x:t>The operation was canceled.</x:t>
   </x:si>
   <x:si>
     <x:t>TC2</x:t>
   </x:si>
   <x:si>
-    <x:t>Test case 'TC2' requires student SERVER but none was found. Grade_Content='Server'</x:t>
-  </x:si>
-  <x:si>
     <x:t>TC3</x:t>
   </x:si>
   <x:si>
-    <x:t>Test case 'TC3' requires student SERVER but none was found. Grade_Content='Server'</x:t>
-  </x:si>
-  <x:si>
     <x:t>TC4</x:t>
   </x:si>
   <x:si>
-    <x:t>Test case 'TC4' requires student SERVER but none was found. Grade_Content='Server'</x:t>
-  </x:si>
-  <x:si>
     <x:t>TC5</x:t>
   </x:si>
   <x:si>
-    <x:t>Test case 'TC5' requires student SERVER but none was found. Grade_Content='Server'</x:t>
-  </x:si>
-  <x:si>
     <x:t>TC6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Test case 'TC6' requires student SERVER but none was found. Grade_Content='Server'</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -440,7 +425,7 @@
     <x:col min="2" max="2" width="7.282054" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="11.853482" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="9.567768" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="77.567768" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="26.282054" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:5" s="1" customFormat="1">
@@ -491,12 +476,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>6</x:v>
@@ -508,12 +493,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>6</x:v>
@@ -525,12 +510,12 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>6</x:v>
@@ -542,12 +527,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>6</x:v>
@@ -559,7 +544,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>